<commit_message>
Add Furnix transfer price markup
</commit_message>
<xml_diff>
--- a/Cabinet_Parts_Price_Parameters_v03.xlsx
+++ b/Cabinet_Parts_Price_Parameters_v03.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PARAMETERS" sheetId="1" r:id="Rd943df28953649b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PARAMETERS" sheetId="1" r:id="Rd500434c25074fa6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,9 +13,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0.0000"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
+    <x:numFmt numFmtId="202" formatCode="0.00&quot;%&quot;"/>
   </x:numFmts>
   <x:fonts count="3">
     <x:font>
@@ -34,7 +35,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -51,8 +52,18 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="4">
+  <x:borders count="7">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
@@ -75,11 +86,41 @@
         <x:color rgb="FFA6A6A6"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF1F4E78"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FF1F4E78"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF1F4E78"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FF1F4E78"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF1F4E78"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FF1F4E78"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF1F4E78"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF1F4E78"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="38">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -126,11 +167,60 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PriceParametersTable" displayName="PriceParametersTable" ref="A1:C10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="Parameter"/>
+    <x:tableColumn id="2" name="Value"/>
+    <x:tableColumn id="3" name="Unit / rule"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -329,19 +419,19 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="64" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A1" s="9" t="str">
+    <x:row r="1" ht="24" hidden="0" customHeight="1">
+      <x:c r="A1" s="25" t="str">
         <x:v>Parameter</x:v>
       </x:c>
-      <x:c r="B1" s="9" t="str">
+      <x:c r="B1" s="26" t="str">
         <x:v>Value</x:v>
       </x:c>
-      <x:c r="C1" s="9" t="str">
+      <x:c r="C1" s="27" t="str">
         <x:v>Unit / rule</x:v>
       </x:c>
       <x:c r="D1" s="9" t="str">
@@ -349,13 +439,13 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A2" s="16" t="str">
+      <x:c r="A2" s="34" t="str">
         <x:v>BACK rate, EUR/m²</x:v>
       </x:c>
-      <x:c r="B2" s="17" t="n">
+      <x:c r="B2" s="35" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="C2" s="18" t="str">
+      <x:c r="C2" s="22" t="str">
         <x:v>EUR/m²</x:v>
       </x:c>
       <x:c r="D2" s="22" t="str">
@@ -363,13 +453,13 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="66" hidden="0" customHeight="1">
-      <x:c r="A3" s="16" t="str">
+      <x:c r="A3" s="34" t="str">
         <x:v>Processing rate, EUR/m²</x:v>
       </x:c>
-      <x:c r="B3" s="17" t="n">
+      <x:c r="B3" s="35" t="n">
         <x:v>17.04</x:v>
       </x:c>
-      <x:c r="C3" s="18" t="str">
+      <x:c r="C3" s="22" t="str">
         <x:v>EUR/m²</x:v>
       </x:c>
       <x:c r="D3" s="22" t="str">
@@ -377,13 +467,13 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="66" hidden="0" customHeight="1">
-      <x:c r="A4" s="16" t="str">
+      <x:c r="A4" s="34" t="str">
         <x:v>WW material rate, EUR/m²</x:v>
       </x:c>
-      <x:c r="B4" s="17" t="n">
+      <x:c r="B4" s="35" t="n">
         <x:v>8.720350877192983</x:v>
       </x:c>
-      <x:c r="C4" s="18" t="str">
+      <x:c r="C4" s="22" t="str">
         <x:v>EUR/m²</x:v>
       </x:c>
       <x:c r="D4" s="22" t="str">
@@ -391,13 +481,13 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="66" hidden="0" customHeight="1">
-      <x:c r="A5" s="16" t="str">
+      <x:c r="A5" s="34" t="str">
         <x:v>BB material rate, EUR/m²</x:v>
       </x:c>
-      <x:c r="B5" s="17" t="n">
+      <x:c r="B5" s="35" t="n">
         <x:v>7.153333333333333</x:v>
       </x:c>
-      <x:c r="C5" s="18" t="str">
+      <x:c r="C5" s="22" t="str">
         <x:v>EUR/m²</x:v>
       </x:c>
       <x:c r="D5" s="22" t="str">
@@ -405,13 +495,13 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="66" hidden="0" customHeight="1">
-      <x:c r="A6" s="16" t="str">
+      <x:c r="A6" s="34" t="str">
         <x:v>NO material rate, EUR/m²</x:v>
       </x:c>
-      <x:c r="B6" s="17" t="n">
+      <x:c r="B6" s="35" t="n">
         <x:v>8.720350877192983</x:v>
       </x:c>
-      <x:c r="C6" s="18" t="str">
+      <x:c r="C6" s="22" t="str">
         <x:v>EUR/m²</x:v>
       </x:c>
       <x:c r="D6" s="22" t="str">
@@ -419,48 +509,62 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="79.19999694824219" hidden="0" customHeight="1">
-      <x:c r="A7" s="16" t="str">
+      <x:c r="A7" s="34" t="str">
         <x:v>Small part threshold, m²</x:v>
       </x:c>
-      <x:c r="B7" s="17" t="n">
+      <x:c r="B7" s="35" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="C7" s="18" t="str">
-        <x:v>m²</x:v>
+      <x:c r="C7" s="22" t="str">
+        <x:v>m²; surcharge when area &lt; threshold</x:v>
       </x:c>
       <x:c r="D7" s="22" t="str">
         <x:v>Priemoka taikoma, kai detalės plotas mažesnis už šią ribą</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A8" s="16" t="str">
+      <x:c r="A8" s="34" t="str">
         <x:v>Small part surcharge, EUR/unit</x:v>
       </x:c>
-      <x:c r="B8" s="17" t="n">
+      <x:c r="B8" s="35" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C8" s="18" t="str">
-        <x:v>EUR/vnt.</x:v>
+      <x:c r="C8" s="22" t="str">
+        <x:v>EUR/unit</x:v>
       </x:c>
       <x:c r="D8" s="22" t="str">
         <x:v>Priemoka vienai mažai detalei</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="79.19999694824219" hidden="0" customHeight="1">
-      <x:c r="A9" s="19" t="str">
-        <x:v>Output decimals</x:v>
-      </x:c>
-      <x:c r="B9" s="20" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C9" s="21" t="str">
-        <x:v>0–8</x:v>
+      <x:c r="A9" s="34" t="str">
+        <x:v>Furnix markup, %</x:v>
+      </x:c>
+      <x:c r="B9" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>Enter 15 for 15%; applied to Furnix unit cost</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
         <x:v>Savikainos apvalinimas prieš palyginimą ir FPACK sumavimą</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="34" t="str">
+        <x:v>Output decimals</x:v>
+      </x:c>
+      <x:c r="B10" s="37" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>digits after decimal point</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2630466537804c75"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>